<commit_message>
Daily EOD data and reports for 2026-07-29
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260729.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260729.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.36</v>
+        <v>1.355</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.055</v>
+        <v>0.05</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.21%</t>
+          <t>3.83%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>208326.16</v>
+        <v>207560.26</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>8424.959999999999</v>
+        <v>7659.05</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.195</v>
+        <v>2.19</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.055</v>
+        <v>0.05</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.57%</t>
+          <t>2.34%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>153650</v>
+        <v>153300</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>3850</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.98</v>
+        <v>0.985</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-0.045</v>
+        <v>-0.04</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-4.39%</t>
+          <t>-3.90%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>56308.84</v>
+        <v>56596.13</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-2585.61</v>
+        <v>-2298.32</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>60.1</v>
+        <v>60.18</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.73</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.23%</t>
+          <t>1.36%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>665006.5</v>
+        <v>665891.7</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>8077.45</v>
+        <v>8962.65</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>178.96</v>
+        <v>178.66</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.18</v>
+        <v>-0.12</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.10%</t>
+          <t>-0.07%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.755</v>
+        <v>0.76</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.01</v>
+        <v>0.015</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.34%</t>
+          <t>2.01%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>7550</v>
+        <v>7600</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>127.595</v>
+        <v>128.07</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>8.074999999999999</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>6.76%</t>
+          <t>7.15%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>510380</v>
+        <v>512280</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>32300</v>
+        <v>34200</v>
       </c>
     </row>
     <row r="12">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.082</v>
+        <v>0.081</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0</v>
+        <v>-0.001</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-1.22%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>771.78</v>
+        <v>762.37</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0</v>
+        <v>-9.41</v>
       </c>
     </row>
     <row r="15">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>37.89</v>
+        <v>37.94</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.13</v>
+        <v>-0.08</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.34%</t>
+          <t>-0.21%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.67</v>
+        <v>32.74</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.38</v>
+        <v>0.45</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.18%</t>
+          <t>1.39%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42078.96</v>
+        <v>42169.12</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>489.44</v>
+        <v>579.6</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1649834.51</v>
+        <v>1651921.85</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>49242.15</v>
+        <v>51329.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>